<commit_message>
chore: update quiz import template structure to match latest schema requirements
</commit_message>
<xml_diff>
--- a/apps/quiz/static/quiz/quiz_import_template.xlsx
+++ b/apps/quiz/static/quiz/quiz_import_template.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -590,69 +590,6 @@
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t>mcq</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="inlineStr">
-        <is>
-          <t>What is entrepreneurship?</t>
-        </is>
-      </c>
-      <c r="C3" s="3" t="inlineStr">
-        <is>
-          <t>Chapter 1: Introduction</t>
-        </is>
-      </c>
-      <c r="D3" s="3" t="inlineStr">
-        <is>
-          <t>The process of creating value</t>
-        </is>
-      </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>A legal status</t>
-        </is>
-      </c>
-      <c r="F3" s="3" t="inlineStr">
-        <is>
-          <t>A business license</t>
-        </is>
-      </c>
-      <c r="G3" s="3" t="inlineStr">
-        <is>
-          <t>A government certificate</t>
-        </is>
-      </c>
-      <c r="H3" s="3" t="inlineStr"/>
-      <c r="I3" s="3" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
-      <c r="J3" s="3" t="inlineStr">
-        <is>
-          <t>Entrepreneurship fundamentally involves creating value.</t>
-        </is>
-      </c>
-      <c r="K3" s="3" t="inlineStr">
-        <is>
-          <t>easy</t>
-        </is>
-      </c>
-      <c r="L3" s="3" t="inlineStr">
-        <is>
-          <t>Definition, Basics</t>
-        </is>
-      </c>
-      <c r="M3" s="3" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:M1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>